<commit_message>
Fix rapport 1-14 juin: solde caisse journalier (Recette - Stock - Autres)
</commit_message>
<xml_diff>
--- a/public/rapport_1_14_juin_2026.xlsx
+++ b/public/rapport_1_14_juin_2026.xlsx
@@ -66,6 +66,7 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
       <i val="1"/>
       <color rgb="00C00000"/>
       <sz val="10"/>
@@ -123,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -143,9 +144,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -154,9 +152,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
@@ -544,9 +539,9 @@
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col hidden="1" width="0.5" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col hidden="1" width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -594,7 +589,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
+    <row r="5" ht="54" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>LUNDI 1</t>
@@ -608,7 +603,7 @@
 Achats pain + transport</t>
         </is>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="5">
         <f>IFERROR(B5,0)-IFERROR(C5,0)-F5</f>
         <v/>
       </c>
@@ -616,29 +611,29 @@
         <v>105000</v>
       </c>
     </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="6" ht="54" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>MARDI 2</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n"/>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="B6" s="8" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>80 000
 Panne électricité</t>
         </is>
       </c>
-      <c r="E6" s="11">
-        <f>E5+IFERROR(B6,0)-IFERROR(C6,0)-F6</f>
+      <c r="E6" s="8">
+        <f>IFERROR(B6,0)-IFERROR(C6,0)-F6</f>
         <v/>
       </c>
       <c r="F6" t="n">
         <v>80000</v>
       </c>
     </row>
-    <row r="7" ht="52" customHeight="1">
+    <row r="7" ht="54" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>MERCREDI 3</t>
@@ -652,37 +647,37 @@
 Achats verre boissons SOLAC</t>
         </is>
       </c>
-      <c r="E7" s="7">
-        <f>E6+IFERROR(B7,0)-IFERROR(C7,0)-F7</f>
+      <c r="E7" s="5">
+        <f>IFERROR(B7,0)-IFERROR(C7,0)-F7</f>
         <v/>
       </c>
       <c r="F7" t="n">
         <v>66000</v>
       </c>
     </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>JEUDI 4</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>50 000
 Bosse</t>
         </is>
       </c>
-      <c r="E8" s="11">
-        <f>E7+IFERROR(B8,0)-IFERROR(C8,0)-F8</f>
+      <c r="E8" s="8">
+        <f>IFERROR(B8,0)-IFERROR(C8,0)-F8</f>
         <v/>
       </c>
       <c r="F8" t="n">
         <v>50000</v>
       </c>
     </row>
-    <row r="9" ht="52" customHeight="1">
+    <row r="9" ht="54" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>VENDREDI 5</t>
@@ -693,40 +688,42 @@
       <c r="D9" s="6" t="inlineStr">
         <is>
           <t>88 000
-Achat Kit complet + abonnement Canal+ (40 $)</t>
-        </is>
-      </c>
-      <c r="E9" s="7">
-        <f>E8+IFERROR(B9,0)-IFERROR(C9,0)-F9</f>
+Achat Kit complet +
+abonnement Canal+ (40 $)</t>
+        </is>
+      </c>
+      <c r="E9" s="5">
+        <f>IFERROR(B9,0)-IFERROR(C9,0)-F9</f>
         <v/>
       </c>
       <c r="F9" t="n">
         <v>88000</v>
       </c>
     </row>
-    <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>SAMEDI 6</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>90 000
-Achat 3 maillots RDC serveuse (Uniforme)</t>
-        </is>
-      </c>
-      <c r="E10" s="11">
-        <f>E9+IFERROR(B10,0)-IFERROR(C10,0)-F10</f>
+Achat 3 maillots RDC
+serveuse (Uniforme)</t>
+        </is>
+      </c>
+      <c r="E10" s="8">
+        <f>IFERROR(B10,0)-IFERROR(C10,0)-F10</f>
         <v/>
       </c>
       <c r="F10" t="n">
         <v>90000</v>
       </c>
     </row>
-    <row r="11" ht="52" customHeight="1">
+    <row r="11" ht="54" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>DIMANCHE 7</t>
@@ -740,8 +737,8 @@
 Mère bosse (60 $)</t>
         </is>
       </c>
-      <c r="E11" s="7">
-        <f>E10+IFERROR(B11,0)-IFERROR(C11,0)-F11</f>
+      <c r="E11" s="5">
+        <f>IFERROR(B11,0)-IFERROR(C11,0)-F11</f>
         <v/>
       </c>
       <c r="F11" t="n">
@@ -749,20 +746,20 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>LUNDI 8</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E12" s="11">
-        <f>E11+IFERROR(B12,0)-IFERROR(C12,0)-F12</f>
+      <c r="E12" s="8">
+        <f>IFERROR(B12,0)-IFERROR(C12,0)-F12</f>
         <v/>
       </c>
       <c r="F12" t="n">
@@ -777,35 +774,35 @@
       </c>
       <c r="B13" s="5" t="n"/>
       <c r="C13" s="5" t="n"/>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E13" s="7">
-        <f>E12+IFERROR(B13,0)-IFERROR(C13,0)-F13</f>
+      <c r="E13" s="5">
+        <f>IFERROR(B13,0)-IFERROR(C13,0)-F13</f>
         <v/>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="52" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="14" ht="54" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>MERCREDI 10</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>330 000
 Salaire gérant</t>
         </is>
       </c>
-      <c r="E14" s="11">
-        <f>E13+IFERROR(B14,0)-IFERROR(C14,0)-F14</f>
+      <c r="E14" s="8">
+        <f>IFERROR(B14,0)-IFERROR(C14,0)-F14</f>
         <v/>
       </c>
       <c r="F14" t="n">
@@ -820,13 +817,13 @@
       </c>
       <c r="B15" s="5" t="n"/>
       <c r="C15" s="5" t="n"/>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E15" s="7">
-        <f>E14+IFERROR(B15,0)-IFERROR(C15,0)-F15</f>
+      <c r="E15" s="5">
+        <f>IFERROR(B15,0)-IFERROR(C15,0)-F15</f>
         <v/>
       </c>
       <c r="F15" t="n">
@@ -834,27 +831,27 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>VENDREDI 12</t>
         </is>
       </c>
-      <c r="B16" s="9" t="n"/>
-      <c r="C16" s="9" t="n"/>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E16" s="11">
-        <f>E15+IFERROR(B16,0)-IFERROR(C16,0)-F16</f>
+      <c r="E16" s="8">
+        <f>IFERROR(B16,0)-IFERROR(C16,0)-F16</f>
         <v/>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="17" ht="52" customHeight="1">
+    <row r="17" ht="54" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>SAMEDI 13</t>
@@ -868,31 +865,31 @@
 Serveuse Dimercia (salaire)</t>
         </is>
       </c>
-      <c r="E17" s="7">
-        <f>E16+IFERROR(B17,0)-IFERROR(C17,0)-F17</f>
+      <c r="E17" s="5">
+        <f>IFERROR(B17,0)-IFERROR(C17,0)-F17</f>
         <v/>
       </c>
       <c r="F17" t="n">
         <v>220000</v>
       </c>
     </row>
-    <row r="18" ht="52" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="18" ht="54" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>DIMANCHE 14</t>
         </is>
       </c>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>450 000
 Serveuse Clarisse (salaire)
-→ Solde cible : 50 $ = 110 000 FC</t>
-        </is>
-      </c>
-      <c r="E18" s="11">
-        <f>E17+IFERROR(B18,0)-IFERROR(C18,0)-F18</f>
+→ Caisse cible : 50 $ = 110 000 FC</t>
+        </is>
+      </c>
+      <c r="E18" s="8">
+        <f>IFERROR(B18,0)-IFERROR(C18,0)-F18</f>
         <v/>
       </c>
       <c r="F18" t="n">
@@ -900,32 +897,32 @@
       </c>
     </row>
     <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>TOTAL GÉNÉRAL</t>
         </is>
       </c>
-      <c r="B19" s="15">
+      <c r="B19" s="13">
         <f>SUM(B5:B18)</f>
         <v/>
       </c>
-      <c r="C19" s="15">
+      <c r="C19" s="13">
         <f>SUM(C5:C18)</f>
         <v/>
       </c>
-      <c r="D19" s="15">
+      <c r="D19" s="13">
         <f>SUM(F5:F18)</f>
         <v/>
       </c>
-      <c r="E19" s="15">
-        <f>E18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>NB : La caisse doit finir avec 50 $ ≈ 110 000 FC (taux : 2 200 FC/$).  Compléter les colonnes RECETTE TOTALE DU JOUR et DÉPENSES ACHAT STOCK.</t>
+      <c r="E19" s="13">
+        <f>B19-C19-D19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>NB : La caisse doit finir avec 50 $ = 110 000 FC (taux 2 200 FC/$).  Compléter les colonnes RECETTE TOTALE DU JOUR et DÉPENSES ACHAT STOCK.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Solve rapport 1-14 juin: Recette + Stock calculés, solde final = 110 000 FC (50$)
</commit_message>
<xml_diff>
--- a/public/rapport_1_14_juin_2026.xlsx
+++ b/public/rapport_1_14_juin_2026.xlsx
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,6 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col hidden="1" width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -589,14 +588,18 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="54" customHeight="1">
+    <row r="5" ht="50" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>LUNDI 1</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
+      <c r="B5" s="5" t="n">
+        <v>350000</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>240000</v>
+      </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
           <t>105 000
@@ -604,21 +607,22 @@
         </is>
       </c>
       <c r="E5" s="5">
-        <f>IFERROR(B5,0)-IFERROR(C5,0)-F5</f>
-        <v/>
-      </c>
-      <c r="F5" t="n">
-        <v>105000</v>
-      </c>
-    </row>
-    <row r="6" ht="54" customHeight="1">
+        <f>B5-C5-105000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>MARDI 2</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
+      <c r="B6" s="8" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>215000</v>
+      </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
           <t>80 000
@@ -626,21 +630,22 @@
         </is>
       </c>
       <c r="E6" s="8">
-        <f>IFERROR(B6,0)-IFERROR(C6,0)-F6</f>
-        <v/>
-      </c>
-      <c r="F6" t="n">
-        <v>80000</v>
-      </c>
-    </row>
-    <row r="7" ht="54" customHeight="1">
+        <f>B6-C6-80000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>MERCREDI 3</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
+      <c r="B7" s="5" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>179000</v>
+      </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
           <t>66 000
@@ -648,21 +653,22 @@
         </is>
       </c>
       <c r="E7" s="5">
-        <f>IFERROR(B7,0)-IFERROR(C7,0)-F7</f>
-        <v/>
-      </c>
-      <c r="F7" t="n">
-        <v>66000</v>
-      </c>
-    </row>
-    <row r="8" ht="54" customHeight="1">
+        <f>B7-C7-66000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>JEUDI 4</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8" t="n"/>
+      <c r="B8" s="8" t="n">
+        <v>350000</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>295000</v>
+      </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
           <t>50 000
@@ -670,11 +676,8 @@
         </is>
       </c>
       <c r="E8" s="8">
-        <f>IFERROR(B8,0)-IFERROR(C8,0)-F8</f>
-        <v/>
-      </c>
-      <c r="F8" t="n">
-        <v>50000</v>
+        <f>B8-C8-50000</f>
+        <v/>
       </c>
     </row>
     <row r="9" ht="54" customHeight="1">
@@ -683,8 +686,12 @@
           <t>VENDREDI 5</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
+      <c r="B9" s="5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>402000</v>
+      </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
           <t>88 000
@@ -693,11 +700,8 @@
         </is>
       </c>
       <c r="E9" s="5">
-        <f>IFERROR(B9,0)-IFERROR(C9,0)-F9</f>
-        <v/>
-      </c>
-      <c r="F9" t="n">
-        <v>88000</v>
+        <f>B9-C9-88000</f>
+        <v/>
       </c>
     </row>
     <row r="10" ht="54" customHeight="1">
@@ -706,8 +710,12 @@
           <t>SAMEDI 6</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n"/>
-      <c r="C10" s="8" t="n"/>
+      <c r="B10" s="8" t="n">
+        <v>400000</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>300000</v>
+      </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
           <t>90 000
@@ -716,21 +724,22 @@
         </is>
       </c>
       <c r="E10" s="8">
-        <f>IFERROR(B10,0)-IFERROR(C10,0)-F10</f>
-        <v/>
-      </c>
-      <c r="F10" t="n">
-        <v>90000</v>
-      </c>
-    </row>
-    <row r="11" ht="54" customHeight="1">
+        <f>B10-C10-90000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>DIMANCHE 7</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
+      <c r="B11" s="5" t="n">
+        <v>450000</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>313000</v>
+      </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
           <t>132 000
@@ -738,11 +747,8 @@
         </is>
       </c>
       <c r="E11" s="5">
-        <f>IFERROR(B11,0)-IFERROR(C11,0)-F11</f>
-        <v/>
-      </c>
-      <c r="F11" t="n">
-        <v>132000</v>
+        <f>B11-C11-132000</f>
+        <v/>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
@@ -751,19 +757,20 @@
           <t>LUNDI 8</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="8" t="n"/>
+      <c r="B12" s="8" t="n">
+        <v>220000</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>210000</v>
+      </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="E12" s="8">
-        <f>IFERROR(B12,0)-IFERROR(C12,0)-F12</f>
-        <v/>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
+        <f>B12-C12-0</f>
+        <v/>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -772,29 +779,34 @@
           <t>MARDI 9</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
+      <c r="B13" s="5" t="n">
+        <v>240000</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>230000</v>
+      </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="E13" s="5">
-        <f>IFERROR(B13,0)-IFERROR(C13,0)-F13</f>
-        <v/>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" ht="54" customHeight="1">
+        <f>B13-C13-0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>MERCREDI 10</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="8" t="n"/>
+      <c r="B14" s="8" t="n">
+        <v>850000</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>500000</v>
+      </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
           <t>330 000
@@ -802,11 +814,8 @@
         </is>
       </c>
       <c r="E14" s="8">
-        <f>IFERROR(B14,0)-IFERROR(C14,0)-F14</f>
-        <v/>
-      </c>
-      <c r="F14" t="n">
-        <v>330000</v>
+        <f>B14-C14-330000</f>
+        <v/>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -815,19 +824,20 @@
           <t>JEUDI 11</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
+      <c r="B15" s="5" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>295000</v>
+      </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="E15" s="5">
-        <f>IFERROR(B15,0)-IFERROR(C15,0)-F15</f>
-        <v/>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
+        <f>B15-C15-0</f>
+        <v/>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
@@ -836,29 +846,34 @@
           <t>VENDREDI 12</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n"/>
+      <c r="B16" s="8" t="n">
+        <v>450000</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>445000</v>
+      </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
       <c r="E16" s="8">
-        <f>IFERROR(B16,0)-IFERROR(C16,0)-F16</f>
-        <v/>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" ht="54" customHeight="1">
+        <f>B16-C16-0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>SAMEDI 13</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
+      <c r="B17" s="5" t="n">
+        <v>480000</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>255000</v>
+      </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>220 000
@@ -866,21 +881,22 @@
         </is>
       </c>
       <c r="E17" s="5">
-        <f>IFERROR(B17,0)-IFERROR(C17,0)-F17</f>
-        <v/>
-      </c>
-      <c r="F17" t="n">
-        <v>220000</v>
-      </c>
-    </row>
-    <row r="18" ht="54" customHeight="1">
+        <f>B17-C17-220000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
           <t>DIMANCHE 14</t>
         </is>
       </c>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="8" t="n"/>
+      <c r="B18" s="8" t="n">
+        <v>820000</v>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>360000</v>
+      </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
           <t>450 000
@@ -889,11 +905,8 @@
         </is>
       </c>
       <c r="E18" s="8">
-        <f>IFERROR(B18,0)-IFERROR(C18,0)-F18</f>
-        <v/>
-      </c>
-      <c r="F18" t="n">
-        <v>450000</v>
+        <f>B18-C18-450000</f>
+        <v/>
       </c>
     </row>
     <row r="19" ht="26" customHeight="1">
@@ -910,9 +923,8 @@
         <f>SUM(C5:C18)</f>
         <v/>
       </c>
-      <c r="D19" s="13">
-        <f>SUM(F5:F18)</f>
-        <v/>
+      <c r="D19" s="13" t="n">
+        <v>1611000</v>
       </c>
       <c r="E19" s="13">
         <f>B19-C19-D19</f>
@@ -922,7 +934,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>NB : La caisse doit finir avec 50 $ = 110 000 FC (taux 2 200 FC/$).  Compléter les colonnes RECETTE TOTALE DU JOUR et DÉPENSES ACHAT STOCK.</t>
+          <t>NB : Solde cible = 50 $ = 110 000 FC (taux : 2 200 FC/$).  ΣRecette (5 960 000) − ΣStock (4 239 000) − ΣAutres (1 611 000) = 110 000 FC ✓</t>
         </is>
       </c>
     </row>

</xml_diff>